<commit_message>
feat: nudge messages submit their WhatsApp templates and show Meta's status
Saving a library message (new, edited or imported) submits its text to Meta
through Gallabox as a Marketing template, named after the message
(smo_m1_01); a {placeholder} becomes a template value. The Messages tab
shows each message's status - approved, waiting for Meta, rejected with the
reason, text changed, not submitted - with Submit for approval, counts, a
filter and a chip on the Nudges header, and the whole message text.

Gallabox cannot edit or delete a template, so changed text is a new version
(_v2), and a template whose text no longer matches is never sent. Deleting a
message deletes its template on Meta when META_SYSTEM_USER_TOKEN and
META_WABA_ID are set; otherwise it is listed to delete in Gallabox. A copy
gets its own template. The 54 SMO message files carry notes on templates,
the 24-hour rule and US numbers.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/nudge-messages/SMO-54-follow-up-messages.xlsx
+++ b/docs/nudge-messages/SMO-54-follow-up-messages.xlsx
@@ -8,7 +8,8 @@
   </bookViews>
   <sheets>
     <sheet name="Messages" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="How to fill it in" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Status and limits" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="How to fill it in" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Messages'!$A$1:$O$55</definedName>
@@ -20,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -31,6 +32,9 @@
     <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="3">
@@ -58,7 +62,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -70,6 +74,7 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -3444,6 +3449,120 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:B8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="110" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>Topic</t>
+        </is>
+      </c>
+      <c r="B1" s="5" t="inlineStr">
+        <is>
+          <t>Read before importing</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>WhatsApp templates</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>All 54 templates (smo_m1_01 ... smo_m6_09) were submitted to Meta through Gallabox on 30 Oct 2026: category Marketing, the exact text of each message, no variables, no buttons. Status when submitted: pending approval. Check them in Gallabox &gt; Templates.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Do not change approved text</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>A template sends the text Meta approved. If you change a message's text here or on the Nudges page, its template no longer matches: submit a new template (a new name, e.g. smo_m1_01_v2), put that name in the WhatsApp template column, and wait for approval.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Who gets which</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Customer messaged the bot in the last 24 hours: the message goes as a normal WhatsApp message - no template needed. Last message over 24 hours ago: only the approved template can be sent (WhatsApp's rule for every business).</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>US (+1) numbers</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Meta currently does not deliver Marketing templates to US numbers at all, even approved ones (paused since April 2025, no end date announced). So US customers get these follow-ups only within 24 hours of their last message to the bot. The Nudges setting 'Skip marketing templates to US (+1) numbers' stops wasted sends; turn it off if Meta lifts the restriction.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>Dish names</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>The handoff says the dish names in the text are examples: check them against the live menu before switching the campaign on.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>Festival messages</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>M4-01, M4-04 and M4-08 speak of festivals and occasions in general terms and go in month 4 like the rest, as the handoff lists them. For a real festival (e.g. Diwali), add a separate message with From, Until, Order by and Kitchens filled in.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>Importing</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>Nudges &gt; Messages &gt; Import, choose this file, check, then Import. Importing again updates the messages by ID and changes nothing else. Only the Messages sheet is read.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:B16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>

</xml_diff>